<commit_message>
vault backup: 2026-03-11 21:05:21
</commit_message>
<xml_diff>
--- a/Курсы/Домашняя работа/Домашняя работа 3/Домашняя работа 2.xlsx
+++ b/Курсы/Домашняя работа/Домашняя работа 3/Домашняя работа 2.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\obsidian-dvfu\Курсы\Домашняя работа\Домашняя работа 3\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC34FF90-9450-4D41-87F7-1F69AC01CEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Описание + особенности аудитори" sheetId="1" r:id="rId1"/>
+    <sheet name="Интервью с автором" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +25,118 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+  <si>
+    <t>Вводные курса</t>
+  </si>
+  <si>
+    <t>Название дисциплины</t>
+  </si>
+  <si>
+    <t>Прикладной искусственный интеллект и нейросети в решении инженерных задач</t>
+  </si>
+  <si>
+    <t>Аудитория (для каких студентов)</t>
+  </si>
+  <si>
+    <t>Студенты технических специальностей (3-4 курс бакалавриата / 1 курс магистратуры) направлений: «Мехатроника и робототехника», «Прикладная механика», «Управление в технических системах», «Биотехнологии», «Нефтегазовое дело». Возраст 20-24 года.</t>
+  </si>
+  <si>
+    <t>Длительность курса (ак.ч.)</t>
+  </si>
+  <si>
+    <t>1 семестр</t>
+  </si>
+  <si>
+    <t>гибрид</t>
+  </si>
+  <si>
+    <t>Параметры аудитории</t>
+  </si>
+  <si>
+    <t>Количество студентов</t>
+  </si>
+  <si>
+    <t>Уровень подготовки студентов (знание предмета)</t>
+  </si>
+  <si>
+    <t>Основы программирования (циклы, функции, ООП), основы математического анализа (производные, градиенты), основы линейной алгебры (матрицы, вектора).</t>
+  </si>
+  <si>
+    <t>Уровень мотивации (желание заниматься)</t>
+  </si>
+  <si>
+    <t>Средний / Ситуативно-высокий.
+Можно выделить три группы:
+1. Энтузиасты (20-30%): Высокая мотивация. Сами читают статьи про ИИ, хотят сделать крутой диплом. Им нужно давать продвинутые задания, чтобы не заскучали.
+2. Прагматики (50-60%): Средняя мотивация. Понимают, что навыки работы с данными повысят их стоимость на рынке труда и помогут с трудоустройством. Будут работать ровно столько, сколько нужно для хорошей оценки и понятного проекта в портфолио.
+3. Слушатели (10-20%): Мотивация низкая. Пришли, потому что «вставили в учебный план» или в магистратуре это обязательный спецкурс. Важно зацепить их интересными практическими кейсами</t>
+  </si>
+  <si>
+    <t>Уровень технической подготовки (владение цифровыми инструментами и сервисами)</t>
+  </si>
+  <si>
+    <t>Базовый / Пользовательский +.
+• Hard skills: Уверенно пользуются Windows, офисным пакетом, браузерами. Знакомы с интерфейсом сред разработки (например, PyCharm, VS Code или Jupyter Notebook), но могли не работать с ними регулярно.
+• Софт: Знают, что такое GitHub (некоторые даже умеют клонировать репозиторий), но с системами контроля версий на постоянной основе не работали.
+• Специфика: Проблема в том, что навык работы с командной строкой / терминалом Linux развит слабо (если это не направление "Информатика"). Это может стать узким местом при развертывании моделей.
+• Главный разрыв: Умеют решать интегралы на бумаге, но теряются, когда ту же задачу нужно запрограммировать.</t>
+  </si>
+  <si>
+    <t>Дополнительные примечания, особенности аудитории</t>
+  </si>
+  <si>
+    <t>1. Высокая загрузка. У студентов технических специальностей очень плотный график: лабораторные, расчетные работы, курсовые по профильным предметам (сопромат, теория машин и механизмов, электротехника). Курс по ИИ не должен быть "второстепенным", но и перегружать их домашними заданиями на 5 часов в день — значит обречь его на провал.
+2. Прагматизм vs. Исследовательский интерес. Им важна прикладная ценность. Фраза "это поможет вам в дипломе" работает лучше, чем "это расширит кругозор".
+3. Языковой барьер. Документация к библиотекам (PyTorch, TensorFlow) и лучшие статьи выходят на английском. Уровень английского у студентов технических специальностей часто средний (читают со словарем). Хорошим тоном будет давать глоссарий терминов на русском.
+4. Боязнь "чистого листа". При работе с кодом многие испытывают ступор перед пустым файлом. Им нужны стартовые шаблоны (темплейты) кода, от которых можно отталкиваться.</t>
+  </si>
+  <si>
+    <t>Среда (онлайн / оффлайн / гибрид)</t>
+  </si>
+  <si>
+    <t>Блок</t>
+  </si>
+  <si>
+    <t>Чек-лист</t>
+  </si>
+  <si>
+    <t>Место для заполнения</t>
+  </si>
+  <si>
+    <t>Интервью с автором</t>
+  </si>
+  <si>
+    <t>Зачем автору реализация данного курса? Какова общая задача курса? Какие образовательные цели программы закрывает данный курс?</t>
+  </si>
+  <si>
+    <t>Каковы будут последствия если слушатели не пройдут данный курс?</t>
+  </si>
+  <si>
+    <t>Какие конкретно навыки/знания должны появиться в руках студентов после завершения данного курса?</t>
+  </si>
+  <si>
+    <t>Какие темы, касающиеся данного курса, студенты уже должны освоить в рамках других дисциплин/курсов?</t>
+  </si>
+  <si>
+    <t>Какие темы необходимо поднять в рамках курса, чтобы студенты могли перейти к изучению других курсов, связанных с данным?</t>
+  </si>
+  <si>
+    <t>Оцените сложность обучения и подчеркните основные "подводные камни", с которыми могут столкнуться обучающиеся</t>
+  </si>
+  <si>
+    <t>Каковы ожидания от результатов обучающихся?</t>
+  </si>
+  <si>
+    <t>Какие сложности могут возникнуть при работе с данной группой (целевой аудиторией)?</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +144,66 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6DCE4"/>
+        <bgColor rgb="FFD6DCE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBBCDFF"/>
+        <bgColor rgb="FFBBCDFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -45,15 +211,121 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +602,190 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="39.28515625" customWidth="1"/>
+    <col min="2" max="2" width="85.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:2" ht="40.5">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="121.5">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="20.25">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="40.5">
+      <c r="A5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="19.5" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="5"/>
+    </row>
+    <row r="7" spans="1:2" ht="20.25">
+      <c r="A7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="81">
+      <c r="A8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="303.75">
+      <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="303.75">
+      <c r="A10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="405">
+      <c r="A11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D95ABB7-729F-47F6-AE50-71CE284C9C58}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18">
+      <c r="A1" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="75.75">
+      <c r="A2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:3" ht="45.75">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="7"/>
+    </row>
+    <row r="4" spans="1:3" ht="60.75">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:3" ht="60.75">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" spans="1:3" ht="60.75">
+      <c r="A6" s="8"/>
+      <c r="B6" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="7"/>
+    </row>
+    <row r="7" spans="1:3" ht="60.75">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="7"/>
+    </row>
+    <row r="8" spans="1:3" ht="30.75">
+      <c r="A8" s="8"/>
+      <c r="B8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="7"/>
+    </row>
+    <row r="9" spans="1:3" ht="45.75">
+      <c r="A9" s="10"/>
+      <c r="B9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>